<commit_message>
Update apartment registry to corrected version
Replace data/apartments.xlsx with the fixed registry: 42 flats with a single
ХВС/ГВС, 38 with split metering (2+2), no mixed flats.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RKvr3FZKXdkS9sqrem757b
</commit_message>
<xml_diff>
--- a/data/apartments.xlsx
+++ b/data/apartments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ОБУЧЕНИЕ\Подборка для создания агента для старшей\БОТ сборщик показаний\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280223EB-3523-4E81-8051-4E38368D174F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CFBF598-4905-4AE0-85BC-961CA1BA6B92}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -308,13 +308,6 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -325,6 +318,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -631,34 +631,34 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="22" style="19" customWidth="1"/>
+    <col min="2" max="2" width="22" style="16" customWidth="1"/>
     <col min="3" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
     </row>
     <row r="2" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
+      <c r="A2" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="13" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -675,7 +675,7 @@
       <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="5">
@@ -692,7 +692,7 @@
       <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C5" s="3">
@@ -709,7 +709,7 @@
       <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C6" s="3">
@@ -726,7 +726,7 @@
       <c r="A7" s="2">
         <v>4</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="5">
@@ -743,7 +743,7 @@
       <c r="A8" s="2">
         <v>5</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="5">
@@ -760,7 +760,7 @@
       <c r="A9" s="2">
         <v>6</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C9" s="3">
@@ -777,7 +777,7 @@
       <c r="A10" s="2">
         <v>7</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="15" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="3">
@@ -794,7 +794,7 @@
       <c r="A11" s="2">
         <v>8</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="5">
@@ -811,7 +811,7 @@
       <c r="A12" s="2">
         <v>9</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="5">
@@ -828,7 +828,7 @@
       <c r="A13" s="2">
         <v>10</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="3">
@@ -845,7 +845,7 @@
       <c r="A14" s="2">
         <v>11</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C14" s="3">
@@ -862,7 +862,7 @@
       <c r="A15" s="2">
         <v>12</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="5">
@@ -879,7 +879,7 @@
       <c r="A16" s="2">
         <v>13</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="5">
@@ -896,7 +896,7 @@
       <c r="A17" s="2">
         <v>14</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C17" s="3">
@@ -913,14 +913,14 @@
       <c r="A18" s="4">
         <v>15</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C18" s="3">
         <v>1</v>
       </c>
       <c r="D18" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18" s="5">
         <v>1</v>
@@ -930,7 +930,7 @@
       <c r="A19" s="4">
         <v>16</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C19" s="5">
@@ -947,7 +947,7 @@
       <c r="A20" s="4">
         <v>17</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="5">
@@ -964,14 +964,14 @@
       <c r="A21" s="4">
         <v>18</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="14" t="s">
         <v>25</v>
       </c>
       <c r="C21" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="5">
         <v>1</v>
@@ -981,7 +981,7 @@
       <c r="A22" s="4">
         <v>19</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="14" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="5">
@@ -998,7 +998,7 @@
       <c r="A23" s="4">
         <v>20</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="5">
@@ -1015,14 +1015,14 @@
       <c r="A24" s="2">
         <v>21</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="3">
         <v>1</v>
@@ -1032,7 +1032,7 @@
       <c r="A25" s="2">
         <v>22</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C25" s="3">
@@ -1049,7 +1049,7 @@
       <c r="A26" s="2">
         <v>23</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C26" s="3">
@@ -1066,14 +1066,14 @@
       <c r="A27" s="2">
         <v>24</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C27" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E27" s="3">
         <v>1</v>
@@ -1083,14 +1083,14 @@
       <c r="A28" s="2">
         <v>25</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C28" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="3">
         <v>1</v>
@@ -1100,7 +1100,7 @@
       <c r="A29" s="2">
         <v>26</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C29" s="3">
@@ -1117,7 +1117,7 @@
       <c r="A30" s="2">
         <v>27</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C30" s="3">
@@ -1134,14 +1134,14 @@
       <c r="A31" s="2">
         <v>28</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C31" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="3">
         <v>1</v>
@@ -1151,14 +1151,14 @@
       <c r="A32" s="2">
         <v>29</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C32" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" s="3">
         <v>1</v>
@@ -1168,7 +1168,7 @@
       <c r="A33" s="2">
         <v>30</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C33" s="3">
@@ -1185,7 +1185,7 @@
       <c r="A34" s="2">
         <v>31</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C34" s="3">
@@ -1202,14 +1202,14 @@
       <c r="A35" s="2">
         <v>32</v>
       </c>
-      <c r="B35" s="18" t="s">
+      <c r="B35" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C35" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E35" s="3">
         <v>1</v>
@@ -1219,14 +1219,14 @@
       <c r="A36" s="2">
         <v>33</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C36" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" s="3">
         <v>1</v>
@@ -1236,7 +1236,7 @@
       <c r="A37" s="2">
         <v>34</v>
       </c>
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C37" s="3">
@@ -1253,7 +1253,7 @@
       <c r="A38" s="2">
         <v>35</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="B38" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C38" s="3">
@@ -1270,14 +1270,14 @@
       <c r="A39" s="2">
         <v>36</v>
       </c>
-      <c r="B39" s="18" t="s">
+      <c r="B39" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C39" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39" s="3">
         <v>1</v>
@@ -1287,14 +1287,14 @@
       <c r="A40" s="2">
         <v>37</v>
       </c>
-      <c r="B40" s="18" t="s">
+      <c r="B40" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C40" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" s="3">
         <v>1</v>
@@ -1304,7 +1304,7 @@
       <c r="A41" s="2">
         <v>38</v>
       </c>
-      <c r="B41" s="18" t="s">
+      <c r="B41" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C41" s="3">
@@ -1321,7 +1321,7 @@
       <c r="A42" s="2">
         <v>39</v>
       </c>
-      <c r="B42" s="18" t="s">
+      <c r="B42" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C42" s="3">
@@ -1338,14 +1338,14 @@
       <c r="A43" s="2">
         <v>40</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C43" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E43" s="3">
         <v>1</v>
@@ -1355,7 +1355,7 @@
       <c r="A44" s="4">
         <v>41</v>
       </c>
-      <c r="B44" s="17" t="s">
+      <c r="B44" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C44" s="5">
@@ -1372,14 +1372,14 @@
       <c r="A45" s="4">
         <v>42</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="B45" s="14" t="s">
         <v>25</v>
       </c>
       <c r="C45" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E45" s="5">
         <v>1</v>
@@ -1389,14 +1389,14 @@
       <c r="A46" s="4">
         <v>43</v>
       </c>
-      <c r="B46" s="17" t="s">
+      <c r="B46" s="14" t="s">
         <v>30</v>
       </c>
       <c r="C46" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D46" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46" s="5">
         <v>1</v>
@@ -1406,7 +1406,7 @@
       <c r="A47" s="4">
         <v>44</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B47" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C47" s="5">
@@ -1423,7 +1423,7 @@
       <c r="A48" s="4">
         <v>45</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="B48" s="14" t="s">
         <v>7</v>
       </c>
       <c r="C48" s="5">
@@ -1440,14 +1440,14 @@
       <c r="A49" s="4">
         <v>46</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B49" s="14" t="s">
         <v>25</v>
       </c>
       <c r="C49" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" s="5">
         <v>1</v>
@@ -1457,7 +1457,7 @@
       <c r="A50" s="2">
         <v>47</v>
       </c>
-      <c r="B50" s="18" t="s">
+      <c r="B50" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C50" s="3">
@@ -1474,7 +1474,7 @@
       <c r="A51" s="2">
         <v>48</v>
       </c>
-      <c r="B51" s="18" t="s">
+      <c r="B51" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C51" s="3">
@@ -1491,14 +1491,14 @@
       <c r="A52" s="2">
         <v>49</v>
       </c>
-      <c r="B52" s="18" t="s">
+      <c r="B52" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C52" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D52" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" s="3">
         <v>1</v>
@@ -1508,7 +1508,7 @@
       <c r="A53" s="2">
         <v>50</v>
       </c>
-      <c r="B53" s="18" t="s">
+      <c r="B53" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C53" s="3">
@@ -1525,7 +1525,7 @@
       <c r="A54" s="2">
         <v>51</v>
       </c>
-      <c r="B54" s="18" t="s">
+      <c r="B54" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C54" s="3">
@@ -1542,7 +1542,7 @@
       <c r="A55" s="2">
         <v>52</v>
       </c>
-      <c r="B55" s="18" t="s">
+      <c r="B55" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C55" s="3">
@@ -1559,7 +1559,7 @@
       <c r="A56" s="2">
         <v>53</v>
       </c>
-      <c r="B56" s="18" t="s">
+      <c r="B56" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C56" s="3">
@@ -1576,7 +1576,7 @@
       <c r="A57" s="2">
         <v>54</v>
       </c>
-      <c r="B57" s="18" t="s">
+      <c r="B57" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C57" s="3">
@@ -1593,7 +1593,7 @@
       <c r="A58" s="2">
         <v>55</v>
       </c>
-      <c r="B58" s="18" t="s">
+      <c r="B58" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C58" s="3">
@@ -1610,14 +1610,14 @@
       <c r="A59" s="2">
         <v>56</v>
       </c>
-      <c r="B59" s="18" t="s">
+      <c r="B59" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C59" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E59" s="3">
         <v>1</v>
@@ -1627,14 +1627,14 @@
       <c r="A60" s="2">
         <v>57</v>
       </c>
-      <c r="B60" s="18" t="s">
+      <c r="B60" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C60" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D60" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E60" s="3">
         <v>1</v>
@@ -1644,7 +1644,7 @@
       <c r="A61" s="2">
         <v>58</v>
       </c>
-      <c r="B61" s="18" t="s">
+      <c r="B61" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C61" s="3">
@@ -1661,7 +1661,7 @@
       <c r="A62" s="2">
         <v>59</v>
       </c>
-      <c r="B62" s="18" t="s">
+      <c r="B62" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C62" s="3">
@@ -1678,14 +1678,14 @@
       <c r="A63" s="2">
         <v>60</v>
       </c>
-      <c r="B63" s="18" t="s">
+      <c r="B63" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C63" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D63" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63" s="3">
         <v>1</v>
@@ -1695,14 +1695,14 @@
       <c r="A64" s="2">
         <v>61</v>
       </c>
-      <c r="B64" s="18" t="s">
+      <c r="B64" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C64" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E64" s="3">
         <v>1</v>
@@ -1712,7 +1712,7 @@
       <c r="A65" s="2">
         <v>62</v>
       </c>
-      <c r="B65" s="18" t="s">
+      <c r="B65" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C65" s="3">
@@ -1729,7 +1729,7 @@
       <c r="A66" s="2">
         <v>63</v>
       </c>
-      <c r="B66" s="18" t="s">
+      <c r="B66" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C66" s="3">
@@ -1746,14 +1746,14 @@
       <c r="A67" s="2">
         <v>64</v>
       </c>
-      <c r="B67" s="18" t="s">
+      <c r="B67" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C67" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D67" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E67" s="3">
         <v>1</v>
@@ -1763,14 +1763,14 @@
       <c r="A68" s="2">
         <v>65</v>
       </c>
-      <c r="B68" s="18" t="s">
+      <c r="B68" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C68" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D68" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E68" s="3">
         <v>1</v>
@@ -1780,7 +1780,7 @@
       <c r="A69" s="2">
         <v>66</v>
       </c>
-      <c r="B69" s="18" t="s">
+      <c r="B69" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C69" s="3">
@@ -1797,7 +1797,7 @@
       <c r="A70" s="2">
         <v>67</v>
       </c>
-      <c r="B70" s="18" t="s">
+      <c r="B70" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C70" s="3">
@@ -1814,14 +1814,14 @@
       <c r="A71" s="2">
         <v>68</v>
       </c>
-      <c r="B71" s="18" t="s">
+      <c r="B71" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C71" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D71" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" s="3">
         <v>1</v>
@@ -1831,14 +1831,14 @@
       <c r="A72" s="2">
         <v>69</v>
       </c>
-      <c r="B72" s="18" t="s">
+      <c r="B72" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C72" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D72" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72" s="3">
         <v>1</v>
@@ -1848,7 +1848,7 @@
       <c r="A73" s="2">
         <v>70</v>
       </c>
-      <c r="B73" s="18" t="s">
+      <c r="B73" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C73" s="3">
@@ -1865,7 +1865,7 @@
       <c r="A74" s="2">
         <v>71</v>
       </c>
-      <c r="B74" s="18" t="s">
+      <c r="B74" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C74" s="3">
@@ -1882,14 +1882,14 @@
       <c r="A75" s="2">
         <v>72</v>
       </c>
-      <c r="B75" s="18" t="s">
+      <c r="B75" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C75" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D75" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E75" s="3">
         <v>1</v>
@@ -1899,14 +1899,14 @@
       <c r="A76" s="2">
         <v>73</v>
       </c>
-      <c r="B76" s="18" t="s">
+      <c r="B76" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C76" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D76" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E76" s="3">
         <v>1</v>
@@ -1916,7 +1916,7 @@
       <c r="A77" s="2">
         <v>74</v>
       </c>
-      <c r="B77" s="18" t="s">
+      <c r="B77" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C77" s="3">
@@ -1933,7 +1933,7 @@
       <c r="A78" s="2">
         <v>75</v>
       </c>
-      <c r="B78" s="18" t="s">
+      <c r="B78" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C78" s="3">
@@ -1950,14 +1950,14 @@
       <c r="A79" s="2">
         <v>76</v>
       </c>
-      <c r="B79" s="18" t="s">
+      <c r="B79" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C79" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D79" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E79" s="3">
         <v>1</v>
@@ -1967,14 +1967,14 @@
       <c r="A80" s="2">
         <v>77</v>
       </c>
-      <c r="B80" s="18" t="s">
+      <c r="B80" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C80" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D80" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E80" s="3">
         <v>1</v>
@@ -1984,7 +1984,7 @@
       <c r="A81" s="2">
         <v>78</v>
       </c>
-      <c r="B81" s="18" t="s">
+      <c r="B81" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C81" s="3">
@@ -2001,7 +2001,7 @@
       <c r="A82" s="2">
         <v>79</v>
       </c>
-      <c r="B82" s="18" t="s">
+      <c r="B82" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C82" s="3">
@@ -2018,14 +2018,14 @@
       <c r="A83" s="2">
         <v>80</v>
       </c>
-      <c r="B83" s="18" t="s">
+      <c r="B83" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C83" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D83" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E83" s="3">
         <v>1</v>

</xml_diff>